<commit_message>
Reunión con el equipo: respuestas anotadas, plan de mejoras (sección 0 de pendientes) y prompt para el chat nuevo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_012doNezrxW4J745NbynyqEt
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_268_EXP3_FAPS2_40V/contracciones_Video_268_EXP3_FAPS2_40V.xlsx
+++ b/data/processed_data/Video_268_EXP3_FAPS2_40V/contracciones_Video_268_EXP3_FAPS2_40V.xlsx
@@ -778,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL2"/>
+  <dimension ref="A1:BP2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,160 +944,180 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>amplitud_relativa_ic95_pct</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>ttp_ic95_s</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>rt50_ic95_s</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>eventos_junto_al_borde</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
         </is>
@@ -1160,14 +1180,14 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>{'n_eventos': 6, 'fuente_tiempo': 'inicio (onset 10 %) en 6 de 6 eventos; pico en el resto', 'modo_busqueda': 'dirigida', 'trenes':    tren           busqueda  ... inicio_s   fin_s
-0     1  dirigida a 0.1 Hz  ...   12.606  62.611
+          <t>{'n_eventos': 6, 'fuente_tiempo': 'inicio (onset 10 %) en 6 de 6 eventos; pico en el resto', 'modo_busqueda': 'libre', 'trenes':    tren busqueda  ... inicio_s   fin_s
+0     1    libre  ...   12.606  62.611
 [1 rows x 17 columns], 'dudosos': Empty DataFrame
 Columns: []
 Index: [], 'sacados_tiempo_amplitud': Empty DataFrame
 Columns: []
 Index: [], 'grupo_por_evento': array(['estimulados', 'estimulados', 'estimulados', 'estimulados',
-       'estimulados', 'estimulados'], dtype=object), 'tren_por_evento': array([1, 1, 1, 1, 1, 1]), 'estimulados': array([0, 1, 2, 3, 4, 5]), 'estimulados_dudosos': array([], dtype=int64), 'espontaneos': array([], dtype=int64), 'hay_estimulacion': True, 'n_trenes_estimulados': 1, 'tren_principal': 1, 'veredicto': 'enganchado a la frecuencia configurada (0.1 Hz)', 'z': 19.289, 'p_valor': 0.000999000999000999, 'periodo_grilla_s': 9.9782, 'periodo_s': 10.00132, 'periodo_err_s': 0.0023, 'frecuencia_Hz': 0.09999, 'frecuencia_err_Hz': 2.3e-05, 'jitter_s': np.float64(0.00962), 'tolerancia_s': 0.0667, 'n_estimulados': 6, 'n_ranuras': 6, 'tasa_captura_pct': 100.0, 'tren_inicio_s': 12.606, 'tren_fin_s': 62.611, 'jitter_limitado_por_resolucion': True, 'resumen_grupos':          grupo  n  ...  amplitud_mediana_px  amplitud_IQR_px
+       'estimulados', 'estimulados'], dtype=object), 'tren_por_evento': array([1, 1, 1, 1, 1, 1]), 'estimulados': array([0, 1, 2, 3, 4, 5]), 'estimulados_dudosos': array([], dtype=int64), 'espontaneos': array([], dtype=int64), 'hay_estimulacion': True, 'n_trenes_estimulados': 1, 'tren_principal': 1, 'veredicto': 'tren periodico a 0.1000 Hz, no se configuro ninguna frecuencia', 'z': 19.289, 'p_valor': 0.000999000999000999, 'periodo_grilla_s': 9.9758, 'periodo_s': 10.00132, 'periodo_err_s': 0.0023, 'frecuencia_Hz': 0.09999, 'frecuencia_err_Hz': 2.3e-05, 'jitter_s': np.float64(0.00962), 'tolerancia_s': 0.0667, 'n_estimulados': 6, 'n_ranuras': 6, 'tasa_captura_pct': 100.0, 'tren_inicio_s': 12.606, 'tren_fin_s': 62.611, 'jitter_limitado_por_resolucion': True, 'resumen_grupos':          grupo  n  ...  amplitud_mediana_px  amplitud_IQR_px
 0  estimulados  6  ...               1.5469             0.09
 [1 rows x 10 columns], 'espontaneas_instantanea': Empty DataFrame
 Columns: [tiempo_s, intervalo_s, frecuencia_Hz]
@@ -1229,98 +1249,108 @@
           <t>0.5636-0.5973</t>
         </is>
       </c>
-      <c r="AG2" t="n">
-        <v>6</v>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>0.5491-0.603</t>
+        </is>
       </c>
       <c r="AH2" t="n">
-        <v>0</v>
+        <v>1.546850000000006</v>
       </c>
       <c r="AI2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
         <v>2</v>
       </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN2" t="n">
+      <c r="AL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
         <v>0.1008333333333304</v>
       </c>
-      <c r="AO2" t="n">
-        <v>6</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ2" t="n">
+      <c r="AR2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
         <v>2</v>
       </c>
-      <c r="AR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV2" t="n">
+      <c r="AU2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
         </is>
       </c>
-      <c r="AX2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
       <c r="BB2" t="n">
         <v>0</v>
       </c>
       <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
         <v>2</v>
       </c>
-      <c r="BD2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BE2" t="n">
+      <c r="BH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI2" t="n">
         <v>0.5999999999999659</v>
       </c>
-      <c r="BF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="inlineStr">
         <is>
           <t>1.5 s: 6 | 2 s: 6 | 3 s: 6</t>
         </is>
       </c>
-      <c r="BH2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BI2" t="inlineStr">
+      <c r="BL2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM2" t="inlineStr">
         <is>
           <t>6 ev en k=5.846-24.421</t>
         </is>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BN2" t="n">
         <v>0.07635389999996427</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BO2" t="n">
         <v>0.04017845999985895</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BP2" t="n">
         <v>1.900369003695819</v>
       </c>
     </row>
@@ -1531,12 +1561,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>dirigida a 0.1 Hz</t>
+          <t>libre</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>enganchado a la frecuencia configurada (0.1 Hz)</t>
+          <t>tren periodico a 0.1000 Hz, no se configuro ninguna frecuencia</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1761,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1790,6 +1820,16 @@
           <t>junto_al_borde</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>en_promedio</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>reportable</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1806,6 +1846,12 @@
       </c>
       <c r="E2" t="b">
         <v>0</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1824,6 +1870,12 @@
       <c r="E3" t="b">
         <v>0</v>
       </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1841,6 +1893,12 @@
       <c r="E4" t="b">
         <v>0</v>
       </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1858,6 +1916,12 @@
       <c r="E5" t="b">
         <v>0</v>
       </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1875,6 +1939,12 @@
       <c r="E6" t="b">
         <v>0</v>
       </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1891,6 +1961,12 @@
       </c>
       <c r="E7" t="b">
         <v>0</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2473,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2504,85 +2580,105 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>amplitud_relativa_ic95_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ttp_ic95_s</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>rt50_ic95_s</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
@@ -2608,47 +2704,57 @@
           <t>0.5636-0.5973</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>6</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.5491-0.603</t>
+        </is>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1.546850000000006</v>
       </c>
       <c r="H2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
         <v>2</v>
       </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
         <v>0.1008333333333304</v>
       </c>
-      <c r="N2" t="n">
-        <v>6</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
+        <v>6</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
         <v>2</v>
       </c>
-      <c r="Q2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
         </is>
@@ -2674,47 +2780,57 @@
           <t>0.5636-0.5973</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>6</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.5491-0.603</t>
+        </is>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1.546850000000006</v>
       </c>
       <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
         <v>2</v>
       </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
         <v>0.1008333333333304</v>
       </c>
-      <c r="N3" t="n">
-        <v>6</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 101 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
         </is>

</xml_diff>